<commit_message>
UVA Supply Bug Fix
</commit_message>
<xml_diff>
--- a/cds_files/UVA_CDS_2021-2022.xlsx
+++ b/cds_files/UVA_CDS_2021-2022.xlsx
@@ -541,9 +541,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:B5"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -554,10 +556,11 @@
         <v>33214</v>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Percent whose need was met</t>
+          <t>On average, the percentage of need that was met</t>
         </is>
       </c>
       <c r="B5" t="n">

</xml_diff>